<commit_message>
Rename skill to product-selection
The name should describe the domain (选品 / product selection), not one of the
data channels it happens to use. Renamed the skill, its config fallback path,
the MCP clientInfo, and the report footer; README/INSTALL updated to the new
repo name. Regenerated the example report so its footer matches.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/selection_data.xlsx
+++ b/examples/selection_data.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-15T00:33:19Z</t>
+          <t>2026-09-15T00:33:30Z</t>
         </is>
       </c>
     </row>
@@ -5446,7 +5446,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>38756 bytes</t>
+          <t>38869 bytes</t>
         </is>
       </c>
     </row>
@@ -5478,7 +5478,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>43737 bytes</t>
+          <t>43343 bytes</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>40704 chars</t>
+          <t>40400 chars</t>
         </is>
       </c>
     </row>
@@ -5566,7 +5566,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>43737 bytes</t>
+          <t>43343 bytes</t>
         </is>
       </c>
     </row>

</xml_diff>